<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-01 La gouttière et le crayon d'Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-01.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-01.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut dessiner la pluie avec son crayon jaune. À l'école il écoute et range le crayon. Un chuchotement serre son ventre. Le soir, il raconte, puis il dessine la gouttière.</t>
+          <t>La maison boit la pluie par la gouttière. Sur le crayon jaune, un éclat de crayon brille. Aniss veut dessiner la chanson, maintenant. Il coupe papa : les mots se perdent. Il pose la feuille trop vite : le papier boit une goutte. À l'école, sa phrase se cogne à la classe. Il refuse de foncer, attend la tasse, dit la chanson. Merci vécu. Sur la ligne jaune, l'éclat de crayon tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière chante sur le toit. La pluie tape la fenêtre de la cuisine. Une petite flaque brille près des bottes jaunes. Ça sent encore la soupe d'hier. Papa range les cuillères dans le tiroir. Maman essuie la table en bois. La maison est douce, un peu sombre. La pluie fait une vraie chanson, Aniss. Tes bottes jaunes t'attendent près de la porte. En ce moment, Aniss tient son crayon jaune. Le bois est lisse sous ses doigts. Je veux dessiner la pluie. Avec le crayon jaune. Il va dans le cartable. Tu le poses tout seul ? Oui, maman. Aniss glisse le crayon dans la poche. Le cartable sent le papier. On enfile les bottes d'abord. Aniss enfile la botte gauche. La botte est froide, un peu lisse. Elle colle, maman. Tire doucement. Et l'autre maintenant. Aniss enfile la botte droite. Tes deux pieds sont au chaud. On y va ? On y va. Tu dis au revoir à maman ? Au revoir, maman. Au revoir, Aniss. Je t'écoute ce soir. Dehors, la rue brille. Les gouttes tapent le capuchon. L'école sent le savon et le bois des casiers. La classe est claire, malgré la pluie. Un carré d'eau coule sur la vitre. La maîtresse parle près du tableau. Bonjour les enfants. On range les crayons. Bonjour, maîtresse. Aniss écoute. Il sort le crayon jaune. Il le pose dans la boîte, tout droit. Le bois tape un tout petit coup. Merci, Aniss. Vous avez bien écouté. Aniss garde le bruit de la gouttière. Il le gardera pour le dessin, plus tard. Plus tard, quelqu'un s'approche. Une voix parle tout bas, tout près de l'oreille. Aniss sent un malaise. Son ventre se serre, tout petit. Il respire. Il reste près de sa chaise. Il pose les mains à plat. Il se souvient de la cuisine. Le soir, la gouttière chante encore. La porte s'ouvre. Ça sent le cacao. Te voilà, Aniss. Tes bottes sont bien mouillées. Viens. Le cacao est chaud. Aniss pose les bottes près de la flaque. Il s'assoit. Le ventre est encore serré. Il regarde papa. Il regarde maman.</t>
+          <t>La maison boit la pluie par la gouttière. Une goutte glisse sur la vitre de la cuisine. La vapeur du cacao fait un petit nuage. La gouttière fait une vraie chanson, Aniss. Tes bottes jaunes attendent près de la flaque. Une petite flaque brille sous la fenêtre. Papa range les cuillères dans le tiroir. Maman essuie la table en bois. Le bois reste un peu humide sous le torchon. Sur le rebord, le crayon jaune attend. Sur le bois lisse, un éclat de crayon brille. Il est petit, papa. C'est la pluie sur le jaune. Le crayon sent le bois, un peu froid. Je dessine la gouttière, maintenant ! Pendant que je finis la table ? Oui, tout de suite ! En ce moment, Aniss saisit le crayon. Le bois est lisse sous ses doigts. Papa parle à maman, près du tiroir. Le cartable est près de la porte. Oui, avec le capuchon. Papa, la gouttière ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? La chanson va partir. Aniss pose une feuille trop vite. Le papier boit une goutte de la table. Le crayon glisse. La ligne jaune part de travers. Oh. L'éclat de crayon tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le crayon va dans le cartable ? Oui, papa. Aniss glisse le crayon dans la poche. Le cartable sent le papier. On enfile les bottes ? Oui. La botte gauche est froide, un peu lisse. Elle colle, maman. Tire vers toi. La botte droite entre, plus facile. On y va ? On y va. Au revoir, maman. Au revoir, Aniss. Dehors, la rue brille sous les gouttes. Les gouttes tapent le capuchon. L'école sent le savon et le bois des casiers. Un carré d'eau coule sur la vitre de la classe. La maîtresse parle près du tableau. Bonjour les enfants. Bonjour, maîtresse. La gouttière, elle chante ! Ses mots se cognent à ceux de la classe. Personne ne comprend la chanson. Aniss referme la bouche. Il serre le crayon dans sa poche. Le soir, la gouttière reprend sa chanson. La porte s'ouvre. Ça sent le cacao. Te voilà, Aniss. Tes bottes sont mouillées. Viens près de la tasse. Aniss pose les bottes près de la flaque. Il s'assoit. Le ventre est serré, tout petit. Il regarde papa. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière chante sur le toit. La pluie tape la fenêtre de la cuisine. Une petite flaque brille près des bottes jaunes. Ça sent encore la soupe d'hier. Papa range les cuillères dans le tiroir. Maman essuie la table en bois. La maison est douce, un peu sombre. La pluie fait une vraie chanson, Aniss. Tes bottes jaunes t'attendent près de la porte. En ce moment, Aniss tient son crayon jaune. Le bois est lisse sous ses doigts. Je veux dessiner la pluie. Avec le crayon jaune. Il va dans le cartable. Tu le poses tout seul ? Oui, maman. Aniss glisse le crayon dans la poche. Le cartable sent le papier. On enfile les bottes d'abord. Aniss enfile la botte gauche. La botte est froide, un peu lisse. Elle colle, maman. Tire doucement. Et l'autre maintenant. Aniss enfile la botte droite. Tes deux pieds sont au chaud. On y va ? On y va. Tu dis au revoir à maman ? Au revoir, maman. Au revoir, Aniss. Je t'écoute ce soir. Dehors, la rue brille. Les gouttes tapent le capuchon. L'école sent le savon et le bois des casiers. La classe est claire, malgré la pluie. Un carré d'eau coule sur la vitre. La maîtresse parle près du tableau. Bonjour les enfants. On range les crayons. Bonjour, maîtresse. Aniss écoute. Il sort le crayon jaune. Il le pose dans la boîte, tout droit. Le bois tape un tout petit coup. Merci, Aniss. Vous avez bien écouté. Aniss garde le bruit de la gouttière. Il le gardera pour le dessin, plus tard. Plus tard, quelqu'un s'approche. Une voix parle tout bas, tout près de l'oreille. Aniss sent un malaise. Son ventre se serre, tout petit. Il respire. Il reste près de sa chaise. Il pose les mains à plat. Il se souvient de la cuisine. Le soir, la gouttière chante encore. La porte s'ouvre. Ça sent le cacao. Te voilà, Aniss. Tes bottes sont bien mouillées. Viens. Le cacao est chaud. Aniss pose les bottes près de la flaque. Il s'assoit. Le ventre est encore serré. Il regarde papa. Il regarde maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La maison boit la pluie par la gouttière. Une goutte glisse sur la vitre de la cuisine. La vapeur du cacao fait un petit nuage. La gouttière fait une vraie chanson, Aniss. Tes bottes jaunes attendent près de la flaque. Une petite flaque brille sous la fenêtre. Papa range les cuillères dans le tiroir. Maman essuie la table en bois. Le bois reste un peu humide sous le torchon. Sur le rebord, le crayon jaune attend. Sur le bois lisse, un &lt;emphasis level="moderate"&gt;éclat de crayon&lt;/emphasis&gt; brille. Il est petit, papa. C'est la pluie sur le jaune. Le crayon sent le bois, un peu froid. Je dessine la gouttière, maintenant ! Pendant que je finis la table ? Oui, tout de suite ! En ce moment, Aniss saisit le crayon. Le bois est lisse sous ses doigts. Papa parle à maman, près du tiroir. Le cartable est près de la porte. Oui, avec le capuchon. Papa, la gouttière ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? La chanson va partir. Aniss pose une feuille trop vite. Le papier boit une goutte de la table. Le crayon glisse. La ligne jaune part de travers. Oh. L'éclat de crayon tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le crayon va dans le cartable ? Oui, papa. Aniss glisse le crayon dans la poche. Le cartable sent le papier. On enfile les bottes ? Oui. La botte gauche est froide, un peu lisse. Elle colle, maman. Tire vers toi. La botte droite entre, plus facile. On y va ? On y va. Au revoir, maman. Au revoir, Aniss. Dehors, la rue brille sous les gouttes. Les gouttes tapent le capuchon. L'école sent le savon et le bois des casiers. Un carré d'eau coule sur la vitre de la classe. La maîtresse parle près du tableau. Bonjour les enfants. Bonjour, maîtresse. La gouttière, elle chante ! Ses mots se cognent à ceux de la classe. Personne ne comprend la chanson. Aniss referme la bouche. Il serre le crayon dans sa poche. Le soir, la gouttière reprend sa chanson. La porte s'ouvre. Ça sent le cacao. Te voilà, Aniss. Tes bottes sont mouillées. Viens près de la tasse. Aniss pose les bottes près de la flaque. Il s'assoit. Le ventre est serré, tout petit. Il regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Nora est à l'école. La maîtresse parle. Nora aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les crayons. Nora range son crayon. Elle écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Garde ça pour toi. Nora sent un malaise. Son ventre est serré. Le soir, papa l'attend. Nora vient raconter à la maison. Elle dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Papa l'écoute. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. [pause]</t>
+          <t>La maison boit la pluie par la gouttière. Une goutte glisse sur la vitre de la cuisine. La vapeur du cacao fait un petit nuage. La gouttière fait une vraie chanson, Aniss. Tes bottes jaunes attendent près de la flaque. Une petite flaque brille sous la fenêtre. Papa range les cuillères dans le tiroir. Maman essuie la table en bois. Le bois reste un peu humide sous le torchon. Sur le rebord, le crayon jaune attend. Sur le bois lisse, un &lt;emphasis&gt;éclat de crayon&lt;/emphasis&gt; brille. Il est petit, papa. C'est la pluie sur le jaune. Le crayon sent le bois, un peu froid. Je dessine la gouttière, maintenant ! Pendant que je finis la table ? Oui, tout de suite ! En ce moment, Aniss saisit le crayon. Le bois est lisse sous ses doigts. Papa parle à maman, près du tiroir. Le cartable est près de la porte. Oui, avec le capuchon. Papa, la gouttière ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? La chanson va partir. Aniss pose une feuille trop vite. Le papier boit une goutte de la table. Le crayon glisse. La ligne jaune part de travers. Oh. L'éclat de crayon tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le crayon va dans le cartable ? Oui, papa. Aniss glisse le crayon dans la poche. Le cartable sent le papier. On enfile les bottes ? Oui. La botte gauche est froide, un peu lisse. Elle colle, maman. Tire vers toi. La botte droite entre, plus facile. On y va ? On y va. Au revoir, maman. Au revoir, Aniss. Dehors, la rue brille sous les gouttes. Les gouttes tapent le capuchon. L'école sent le savon et le bois des casiers. Un carré d'eau coule sur la vitre de la classe. La maîtresse parle près du tableau. Bonjour les enfants. Bonjour, maîtresse. La gouttière, elle chante ! Ses mots se cognent à ceux de la classe. Personne ne comprend la chanson. Aniss referme la bouche. Il serre le crayon dans sa poche. Le soir, la gouttière reprend sa chanson. La porte s'ouvre. Ça sent le cacao. Te voilà, Aniss. Tes bottes sont mouillées. Viens près de la tasse. Aniss pose les bottes près de la flaque. Il s'assoit. Le ventre est serré, tout petit. Il regarde papa. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de crayon</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,78 +1321,88 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_dessiner_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La gouttière chante sur le toit.
-narrateur|La pluie tape la fenêtre de la cuisine.
-narrateur|Une petite flaque brille près des bottes jaunes.
-narrateur|Ça sent encore la soupe d'hier.
+          <t>narrateur|La maison boit la pluie par la gouttière.
+narrateur|Une goutte glisse sur la vitre de la cuisine.
+narrateur|La vapeur du cacao fait un petit nuage.
+papa|La gouttière fait une vraie chanson, Aniss.
+maman|Tes bottes jaunes attendent près de la flaque.
+narrateur|Une petite flaque brille sous la fenêtre.
 narrateur|Papa range les cuillères dans le tiroir.
 narrateur|Maman essuie la table en bois.
-narrateur|La maison est douce, un peu sombre.
-papa|La pluie fait une vraie chanson, Aniss.
-maman|Tes bottes jaunes t'attendent près de la porte.
-narrateur|En ce moment, Aniss tient son crayon jaune.
+narrateur|Le bois reste un peu humide sous le torchon.
+narrateur|Sur le rebord, le crayon jaune attend.
+narrateur|Sur le bois lisse, un éclat de crayon brille.
+enfant-m|Il est petit, papa.
+papa|C'est la pluie sur le jaune.
+narrateur|Le crayon sent le bois, un peu froid.
+enfant-m|Je dessine la gouttière, maintenant !
+maman|Pendant que je finis la table ?
+enfant-m|Oui, tout de suite !
+narrateur|En ce moment, Aniss saisit le crayon.
 narrateur|Le bois est lisse sous ses doigts.
-enfant-m|Je veux dessiner la pluie.
-enfant-m|Avec le crayon jaune.
-maman|Il va dans le cartable.
-maman|Tu le poses tout seul ?
-enfant-m|Oui, maman.
+narrateur|Papa parle à maman, près du tiroir.
+papa|Le cartable est près de la porte.
+maman|Oui, avec le capuchon.
+enfant-m|Papa, la gouttière !
+narrateur|Les mots d'Aniss se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Aniss ?
+enfant-m|La chanson va partir.
+narrateur|Aniss pose une feuille trop vite.
+narrateur|Le papier boit une goutte de la table.
+narrateur|Le crayon glisse.
+narrateur|La ligne jaune part de travers.
+enfant-m|Oh.
+narrateur|L'éclat de crayon tremble, puis tient.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça ne veut pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Le crayon va dans le cartable ?
+enfant-m|Oui, papa.
 narrateur|Aniss glisse le crayon dans la poche.
 narrateur|Le cartable sent le papier.
-papa|On enfile les bottes d'abord.
-narrateur|Aniss enfile la botte gauche.
-narrateur|La botte est froide, un peu lisse.
+papa|On enfile les bottes ?
+enfant-m|Oui.
+narrateur|La botte gauche est froide, un peu lisse.
 enfant-m|Elle colle, maman.
-maman|Tire doucement.
-maman|Et l'autre maintenant.
-narrateur|Aniss enfile la botte droite.
-papa|Tes deux pieds sont au chaud.
+maman|Tire vers toi.
+narrateur|La botte droite entre, plus facile.
 papa|On y va ?
 enfant-m|On y va.
-papa|Tu dis au revoir à maman ?
 enfant-m|Au revoir, maman.
 maman|Au revoir, Aniss.
-maman|Je t'écoute ce soir.
-narrateur|Dehors, la rue brille.
+narrateur|Dehors, la rue brille sous les gouttes.
 narrateur|Les gouttes tapent le capuchon.
 narrateur|L'école sent le savon et le bois des casiers.
-narrateur|La classe est claire, malgré la pluie.
-narrateur|Un carré d'eau coule sur la vitre.
+narrateur|Un carré d'eau coule sur la vitre de la classe.
 narrateur|La maîtresse parle près du tableau.
 maitresse|Bonjour les enfants.
-maitresse|On range les crayons.
 enfant-m|Bonjour, maîtresse.
-narrateur|Aniss écoute.
-narrateur|Il sort le crayon jaune.
-narrateur|Il le pose dans la boîte, tout droit.
-narrateur|Le bois tape un tout petit coup.
-maitresse|Merci, Aniss.
-maitresse|Vous avez bien écouté.
-narrateur|Aniss garde le bruit de la gouttière.
-narrateur|Il le gardera pour le dessin, plus tard.
-narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, tout près de l'oreille.
-narrateur|Aniss sent un malaise.
-narrateur|Son ventre se serre, tout petit.
-narrateur|Il respire.
-narrateur|Il reste près de sa chaise.
-narrateur|Il pose les mains à plat.
-narrateur|Il se souvient de la cuisine.
-narrateur|Le soir, la gouttière chante encore.
+enfant-m|La gouttière, elle chante !
+narrateur|Ses mots se cognent à ceux de la classe.
+narrateur|Personne ne comprend la chanson.
+narrateur|Aniss referme la bouche.
+narrateur|Il serre le crayon dans sa poche.
+narrateur|Le soir, la gouttière reprend sa chanson.
 narrateur|La porte s'ouvre.
 narrateur|Ça sent le cacao.
 papa|Te voilà, Aniss.
-papa|Tes bottes sont bien mouillées.
-maman|Viens.
-maman|Le cacao est chaud.
+papa|Tes bottes sont mouillées.
+maman|Viens près de la tasse.
 narrateur|Aniss pose les bottes près de la flaque.
 narrateur|Il s'assoit.
-narrateur|Le ventre est encore serré.
+narrateur|Le ventre est serré, tout petit.
 narrateur|Il regarde papa.
-narrateur|Il regarde maman.</t>
+narrateur|Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1424,27 +1434,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Aniss a un malaise. Que fait-il ?</t>
+          <t>Aniss veut dire la chanson. Que fait-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss a un malaise. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss veut dire la &lt;emphasis level="moderate"&gt;chanson&lt;/emphasis&gt;. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nora a un malaise. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss veut dire la &lt;emphasis&gt;chanson&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>raconter</t>
+          <t>il attend</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | il raconte | à papa | à la maison | écouter</t>
+          <t>il attend | attendre | son tour | il écoute | il attend son tour | attendre la fin</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1459,7 +1469,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il raconte à papa. Que fait Aniss ?</t>
+          <t>Papa n'a pas fini sa phrase. Que fait Aniss ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1497,7 +1507,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1508,7 +1518,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1523,34 +1533,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>chanson</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1565,22 +1579,22 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_attend_la_fin_de_la_phrase; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Aniss a un malaise.
+          <t>narrateur|Aniss veut dire la chanson.
 narrateur|Que fait-il ?</t>
         </is>
       </c>
@@ -1608,17 +1622,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa. Maman. J'ai eu un malaise. Quelqu'un a parlé tout bas. On t'écoute. Viens près de la tasse. Aniss parle, tout doucement. Papa écoute sans couper. Maman pose une main tiède sur son dos. Tu as bien fait de venir le dire. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens raconter. Le ventre d'Aniss se desserre, un peu. Tu as fini ta tasse ? Presque, maman.</t>
+          <t>Aniss ouvre la bouche trop vite. Papa, la gouttière. Papa n'a pas fini sa phrase. Le cacao est chaud, Aniss. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il referme la bouche. Il pose les mains à plat. Il écoute la cuisine, un instant. Tes bottes sèchent près de la porte. Papa pose sa tasse. Le cacao fume un peu. Maman n'a pas fini non plus. Aniss attend que le silence arrive. Sur le rebord, l'éclat de crayon brille. Il est là. Je peux te montrer quelque chose ? Oui, nous t'écoutons. La gouttière chante sur le toit. Mon crayon a vu la pluie. Merci, Aniss. Papa a entendu toute la phrase. Tu as fini ta tasse ? Presque, maman. Le ventre d'Aniss se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Papa. Maman. J'ai eu un malaise. Quelqu'un a parlé tout bas. On t'écoute. Viens près de la tasse. Aniss parle, tout doucement. Papa écoute sans couper. Maman pose une main tiède sur son dos. Tu as bien fait de venir le dire. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens raconter. Le ventre d'Aniss se desserre, un peu. Tu as fini ta tasse ? Presque, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss ouvre la bouche trop vite. Papa, la gouttière. Papa n'a pas fini sa phrase. Le cacao est chaud, Aniss. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il referme la bouche. Il pose les mains à plat. Il écoute la cuisine, un instant. Tes bottes sèchent près de la porte. Papa pose sa &lt;emphasis level="moderate"&gt;tasse&lt;/emphasis&gt;. Le cacao fume un peu. Maman n'a pas fini non plus. Aniss attend que le silence arrive. Sur le rebord, l'éclat de crayon brille. Il est là. Je peux te montrer quelque chose ? Oui, nous t'écoutons. La gouttière chante sur le toit. Mon crayon a vu la pluie. Merci, Aniss. Papa a entendu toute la phrase. Tu as fini ta tasse ? Presque, maman. Le ventre d'Aniss se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nora a écouté la maîtresse. Elle a raconté son malaise à la maison. Papa est là. [pause]</t>
+          <t>Aniss ouvre la bouche trop vite. Papa, la gouttière. Papa n'a pas fini sa phrase. Le cacao est chaud, Aniss. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il referme la bouche. Il pose les mains à plat. Il écoute la cuisine, un instant. Tes bottes sèchent près de la porte. Papa pose sa &lt;emphasis&gt;tasse&lt;/emphasis&gt;. Le cacao fume un peu. Maman n'a pas fini non plus. Aniss attend que le silence arrive. Sur le rebord, l'éclat de crayon brille. Il est là. Je peux te montrer quelque chose ? Oui, nous t'écoutons. La gouttière chante sur le toit. Mon crayon a vu la pluie. Merci, Aniss. Papa a entendu toute la phrase. Tu as fini ta tasse ? Presque, maman. Le ventre d'Aniss se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1665,7 +1679,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1673,10 +1687,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1697,28 +1711,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>tasse</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1727,10 +1745,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1743,26 +1761,43 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Papa.
-enfant-m|Maman.
-enfant-m|J'ai eu un malaise.
-enfant-m|Quelqu'un a parlé tout bas.
-papa|On t'écoute.
-maman|Viens près de la tasse.
-narrateur|Aniss parle, tout doucement.
-narrateur|Papa écoute sans couper.
-narrateur|Maman pose une main tiède sur son dos.
-maman|Tu as bien fait de venir le dire.
-papa|À l'école, on écoute la maîtresse.
-papa|Si tu as un malaise, tu viens raconter.
-narrateur|Le ventre d'Aniss se desserre, un peu.
+          <t>narrateur|Aniss ouvre la bouche trop vite.
+enfant-m|Papa, la gouttière.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le cacao est chaud, Aniss.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Aniss refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il pose les mains à plat.
+narrateur|Il écoute la cuisine, un instant.
+papa|Tes bottes sèchent près de la porte.
+narrateur|Papa pose sa tasse.
+maman|Le cacao fume un peu.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Aniss attend que le silence arrive.
+narrateur|Sur le rebord, l'éclat de crayon brille.
+enfant-m|Il est là.
+enfant-m|Je peux te montrer quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|La gouttière chante sur le toit.
+enfant-m|Mon crayon a vu la pluie.
+papa|Merci, Aniss.
+narrateur|Papa a entendu toute la phrase.
 maman|Tu as fini ta tasse ?
-enfant-m|Presque, maman.</t>
+enfant-m|Presque, maman.
+narrateur|Le ventre d'Aniss se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tasse,cacao</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1824,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Aniss sort le crayon jaune du cartable. Le bois est encore un peu froid. Je dessine la gouttière. Tu lui fais une place sur la feuille ? Oui. Ici, au milieu. Aniss trace une ligne jaune, tout long. La ligne descend, comme l'eau. On entend presque la chanson. Aniss ajoute une petite flaque ronde. Et les bottes, à côté ? Deux bottes jaunes. Il souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre.</t>
+          <t>Aniss sort le crayon jaune du cartable. Le bois est froid, un peu lisse. Je dessine la gouttière. Tu lui fais une place sur la feuille ? Oui. Ici, au milieu. Aniss veut tracer tout de suite. Il appuie trop fort. Le papier se plisse. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il écoute la gouttière, un instant. Il reprend le crayon, plus léger. Une ligne jaune descend, comme l'eau. On entend presque la chanson. Aniss ajoute une petite flaque ronde. Et les bottes, à côté ? Deux bottes jaunes. Il souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Aniss sort le crayon jaune du cartable. Le bois est encore un peu froid. Je dessine la gouttière. Tu lui fais une place sur la feuille ? Oui. Ici, au milieu. Aniss trace une ligne jaune, tout long. La ligne descend, comme l'eau. On entend presque la chanson. Aniss ajoute une petite flaque ronde. Et les bottes, à côté ? Deux bottes jaunes. Il souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss sort le crayon jaune du cartable. Le bois est froid, un peu lisse. Je dessine la &lt;emphasis level="moderate"&gt;gouttière&lt;/emphasis&gt;. Tu lui fais une place sur la feuille ? Oui. Ici, au milieu. Aniss veut tracer tout de suite. Il appuie trop fort. Le papier se plisse. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il écoute la gouttière, un instant. Il reprend le crayon, plus léger. Une ligne jaune descend, comme l'eau. On entend presque la chanson. Aniss ajoute une petite flaque ronde. Et les bottes, à côté ? Deux bottes jaunes. Il souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Nora boit un verre d'eau. Papa lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Aniss sort le crayon jaune du cartable. Le bois est froid, un peu lisse. Je dessine la &lt;emphasis&gt;gouttière&lt;/emphasis&gt;. Tu lui fais une place sur la feuille ? Oui. Ici, au milieu. Aniss veut tracer tout de suite. Il appuie trop fort. Le papier se plisse. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il écoute la gouttière, un instant. Il reprend le crayon, plus léger. Une ligne jaune descend, comme l'eau. On entend presque la chanson. Aniss ajoute une petite flaque ronde. Et les bottes, à côté ? Deux bottes jaunes. Il souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,7 +1881,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1854,10 +1889,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1880,30 +1915,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>gouttière</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1912,10 +1947,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1926,17 +1961,29 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_la_feuille; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Aniss sort le crayon jaune du cartable.
-narrateur|Le bois est encore un peu froid.
+narrateur|Le bois est froid, un peu lisse.
 enfant-m|Je dessine la gouttière.
 papa|Tu lui fais une place sur la feuille ?
 enfant-m|Oui.
 enfant-m|Ici, au milieu.
-narrateur|Aniss trace une ligne jaune, tout long.
-narrateur|La ligne descend, comme l'eau.
+narrateur|Aniss veut tracer tout de suite.
+narrateur|Il appuie trop fort.
+narrateur|Le papier se plisse.
+enfant-m|Oh.
+narrateur|Aniss s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il refuse de foncer.
+narrateur|Il écoute la gouttière, un instant.
+narrateur|Il reprend le crayon, plus léger.
+narrateur|Une ligne jaune descend, comme l'eau.
 maman|On entend presque la chanson.
 narrateur|Aniss ajoute une petite flaque ronde.
 papa|Et les bottes, à côté ?
@@ -1946,6 +1993,11 @@
 narrateur|La pluie ralentit derrière la vitre.</t>
         </is>
       </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>crayon,papier</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1970,17 +2022,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les bottes sèchent près de la porte. La feuille jaune reste sur la table. On t'a écouté, Aniss. La gouttière chante encore, plus loin.</t>
+          <t>Les bottes sèchent près de la porte. La feuille jaune reste sur la table. Comme sur le rebord, papa ! Tu le vois, toi ? Oui, sur le jaune. On est bien, ici. Le cacao fume un peu, près de la fenêtre. Aniss glisse le crayon sans se presser. Le bois repose contre la feuille. On l'entend, maman. Tu l'entends sur le papier ? Oui, la chanson. La pluie reste dans l'air. L'éclat de crayon tient sur la ligne.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les bottes sèchent près de la porte. La feuille jaune reste sur la table. On t'a écouté, Aniss. La gouttière chante encore, plus loin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les bottes sèchent près de la porte. La feuille jaune reste sur la table. Comme sur le rebord, papa ! Tu le vois, toi ? Oui, sur le jaune. On est bien, ici. Le cacao fume un peu, près de la fenêtre. Aniss glisse le crayon sans se presser. Le bois repose contre la feuille. On l'entend, maman. Tu l'entends sur le papier ? Oui, la chanson. La pluie reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de crayon&lt;/emphasis&gt; tient sur la ligne.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les bottes sèchent près de la porte. La feuille jaune reste sur la table. Comme sur le rebord, papa ! Tu le vois, toi ? Oui, sur le jaune. On est bien, ici. Le cacao fume un peu, près de la fenêtre. Aniss glisse le crayon sans se presser. Le bois repose contre la feuille. On l'entend, maman. Tu l'entends sur le papier ? Oui, la chanson. La pluie reste dans l'air. L'&lt;emphasis&gt;éclat de crayon&lt;/emphasis&gt; tient sur la ligne.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2027,7 +2079,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2035,10 +2087,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2047,12 +2099,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2061,17 +2113,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de crayon</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2080,11 +2136,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2093,27 +2149,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_ligne; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Les bottes sèchent près de la porte.
 narrateur|La feuille jaune reste sur la table.
-maman|On t'a écouté, Aniss.
-papa|La gouttière chante encore, plus loin.</t>
+enfant-m|Comme sur le rebord, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le jaune.
+maman|On est bien, ici.
+narrateur|Le cacao fume un peu, près de la fenêtre.
+narrateur|Aniss glisse le crayon sans se presser.
+narrateur|Le bois repose contre la feuille.
+enfant-m|On l'entend, maman.
+maman|Tu l'entends sur le papier ?
+enfant-m|Oui, la chanson.
+narrateur|La pluie reste dans l'air.
+narrateur|L'éclat de crayon tient sur la ligne.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>gouttiere,pluie</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2191,6 +2266,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>